<commit_message>
Update importer to cover all 42 of 69 pages
Automated migration updates generated by Experience Modernization Agent.

Changed files (11):
- tools/importer/import-cp-landing-page.bundle.js
- tools/importer/import-cp-landing-page.js
- tools/importer/import-services-detail-page.bundle.js
- tools/importer/import-services-detail-page.js
- tools/importer/page-templates.json
- tools/importer/reports/en-us/lp/dell-experience.report.json
- tools/importer/reports/en-us/lp/dt/automation-platform.report.json
- tools/importer/reports/import-cp-landing-page.report.xlsx
- tools/importer/reports/import-services-detail-page.report.xlsx
- tools/importer/urls-automation-platform.txt
- tools/importer/urls-dell-experience.txt
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-cp-landing-page.report.xlsx
+++ b/tools/importer/reports/import-cp-landing-page.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="226">
   <si>
     <t>_reportFile</t>
   </si>
@@ -43,24 +43,42 @@
     <t>url</t>
   </si>
   <si>
+    <t>en-us/lp/dell-experience.report.json</t>
+  </si>
+  <si>
+    <t>["hero","cards","tabs","carousel","carousel","carousel"]</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>en-us/lp/dell-experience</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>cp-landing-page</t>
+  </si>
+  <si>
+    <t>2026-03-20T20:48:34.819Z</t>
+  </si>
+  <si>
+    <t>Why Buy Direct from Dell | Dell USA</t>
+  </si>
+  <si>
+    <t>https://www.dell.com/en-us/lp/dell-experience</t>
+  </si>
+  <si>
     <t>en-us/lp/dell-video-conferencing-room-solutions.report.json</t>
   </si>
   <si>
     <t>["hero","cards","cards","columns","columns","columns","tabs","tabs","carousel"]</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>en-us/lp/dell-video-conferencing-room-solutions</t>
   </si>
   <si>
-    <t>success</t>
-  </si>
-  <si>
-    <t>cp-landing-page</t>
-  </si>
-  <si>
     <t>2026-03-20T17:13:36.771Z</t>
   </si>
   <si>
@@ -146,6 +164,24 @@
   </si>
   <si>
     <t>https://www.dell.com/en-us/lp/dt/artificial-intelligence-services</t>
+  </si>
+  <si>
+    <t>en-us/lp/dt/automation-platform.report.json</t>
+  </si>
+  <si>
+    <t>["columns","cards","cards","cards","cards","carousel"]</t>
+  </si>
+  <si>
+    <t>en-us/lp/dt/automation-platform</t>
+  </si>
+  <si>
+    <t>2026-03-20T20:48:23.280Z</t>
+  </si>
+  <si>
+    <t>Dell Automation Platform | Dell USA</t>
+  </si>
+  <si>
+    <t>https://www.dell.com/en-us/lp/dt/automation-platform</t>
   </si>
   <si>
     <t>en-us/lp/dt/customer-stories-mclaren-racing.report.json</t>
@@ -1045,7 +1081,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:J36"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="5" width="50" customWidth="1"/>
@@ -1138,39 +1174,39 @@
         <v>14</v>
       </c>
       <c r="G3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" t="s">
         <v>22</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>23</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>24</v>
-      </c>
-      <c r="J3" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" t="s">
         <v>26</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" t="s">
         <v>27</v>
       </c>
-      <c r="C4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G4" t="s">
         <v>28</v>
-      </c>
-      <c r="F4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G4" t="s">
-        <v>22</v>
       </c>
       <c r="H4" t="s">
         <v>29</v>
@@ -1202,7 +1238,7 @@
         <v>14</v>
       </c>
       <c r="G5" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H5" t="s">
         <v>35</v>
@@ -1234,103 +1270,103 @@
         <v>14</v>
       </c>
       <c r="G6" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" t="s">
         <v>41</v>
       </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>42</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" t="s">
         <v>43</v>
-      </c>
-      <c r="J6" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" t="s">
         <v>45</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" t="s">
         <v>46</v>
       </c>
-      <c r="C7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" t="s">
         <v>47</v>
       </c>
-      <c r="F7" t="s">
-        <v>14</v>
-      </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>48</v>
       </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>49</v>
       </c>
-      <c r="I7" t="s">
+      <c r="J7" t="s">
         <v>50</v>
-      </c>
-      <c r="J7" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" t="s">
         <v>52</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" t="s">
         <v>53</v>
       </c>
-      <c r="C8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" t="s">
+        <v>47</v>
+      </c>
+      <c r="H8" t="s">
         <v>54</v>
       </c>
-      <c r="F8" t="s">
-        <v>14</v>
-      </c>
-      <c r="G8" t="s">
-        <v>41</v>
-      </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
         <v>55</v>
       </c>
-      <c r="I8" t="s">
+      <c r="J8" t="s">
         <v>56</v>
-      </c>
-      <c r="J8" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>57</v>
+      </c>
+      <c r="B9" t="s">
         <v>58</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" t="s">
         <v>59</v>
       </c>
-      <c r="C9" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" t="s">
         <v>60</v>
-      </c>
-      <c r="F9" t="s">
-        <v>14</v>
-      </c>
-      <c r="G9" t="s">
-        <v>22</v>
       </c>
       <c r="H9" t="s">
         <v>61</v>
@@ -1362,7 +1398,7 @@
         <v>14</v>
       </c>
       <c r="G10" t="s">
-        <v>22</v>
+        <v>47</v>
       </c>
       <c r="H10" t="s">
         <v>67</v>
@@ -1394,71 +1430,71 @@
         <v>14</v>
       </c>
       <c r="G11" t="s">
+        <v>28</v>
+      </c>
+      <c r="H11" t="s">
         <v>73</v>
       </c>
-      <c r="H11" t="s">
+      <c r="I11" t="s">
         <v>74</v>
       </c>
-      <c r="I11" t="s">
+      <c r="J11" t="s">
         <v>75</v>
-      </c>
-      <c r="J11" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B12" t="s">
         <v>77</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
+        <v>12</v>
+      </c>
+      <c r="D12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" t="s">
         <v>78</v>
       </c>
-      <c r="C12" t="s">
-        <v>12</v>
-      </c>
-      <c r="D12" t="s">
-        <v>12</v>
-      </c>
-      <c r="E12" t="s">
+      <c r="F12" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" t="s">
+        <v>28</v>
+      </c>
+      <c r="H12" t="s">
         <v>79</v>
       </c>
-      <c r="F12" t="s">
-        <v>14</v>
-      </c>
-      <c r="G12" t="s">
-        <v>41</v>
-      </c>
-      <c r="H12" t="s">
+      <c r="I12" t="s">
         <v>80</v>
       </c>
-      <c r="I12" t="s">
+      <c r="J12" t="s">
         <v>81</v>
-      </c>
-      <c r="J12" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>82</v>
+      </c>
+      <c r="B13" t="s">
         <v>83</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" t="s">
         <v>84</v>
       </c>
-      <c r="C13" t="s">
-        <v>12</v>
-      </c>
-      <c r="D13" t="s">
-        <v>12</v>
-      </c>
-      <c r="E13" t="s">
+      <c r="F13" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" t="s">
         <v>85</v>
-      </c>
-      <c r="F13" t="s">
-        <v>14</v>
-      </c>
-      <c r="G13" t="s">
-        <v>41</v>
       </c>
       <c r="H13" t="s">
         <v>86</v>
@@ -1475,7 +1511,7 @@
         <v>89</v>
       </c>
       <c r="B14" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="C14" t="s">
         <v>12</v>
@@ -1484,30 +1520,30 @@
         <v>12</v>
       </c>
       <c r="E14" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F14" t="s">
         <v>14</v>
       </c>
       <c r="G14" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="H14" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I14" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B15" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C15" t="s">
         <v>12</v>
@@ -1516,30 +1552,30 @@
         <v>12</v>
       </c>
       <c r="E15" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F15" t="s">
         <v>14</v>
       </c>
       <c r="G15" t="s">
-        <v>22</v>
+        <v>47</v>
       </c>
       <c r="H15" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="I15" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J15" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B16" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="C16" t="s">
         <v>12</v>
@@ -1554,7 +1590,7 @@
         <v>14</v>
       </c>
       <c r="G16" t="s">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="H16" t="s">
         <v>103</v>
@@ -1586,7 +1622,7 @@
         <v>14</v>
       </c>
       <c r="G17" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="H17" t="s">
         <v>109</v>
@@ -1618,7 +1654,7 @@
         <v>14</v>
       </c>
       <c r="G18" t="s">
-        <v>41</v>
+        <v>85</v>
       </c>
       <c r="H18" t="s">
         <v>115</v>
@@ -1650,24 +1686,24 @@
         <v>14</v>
       </c>
       <c r="G19" t="s">
+        <v>47</v>
+      </c>
+      <c r="H19" t="s">
         <v>121</v>
       </c>
-      <c r="H19" t="s">
+      <c r="I19" t="s">
         <v>122</v>
       </c>
-      <c r="I19" t="s">
+      <c r="J19" t="s">
         <v>123</v>
-      </c>
-      <c r="J19" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>124</v>
+      </c>
+      <c r="B20" t="s">
         <v>125</v>
-      </c>
-      <c r="B20" t="s">
-        <v>71</v>
       </c>
       <c r="C20" t="s">
         <v>12</v>
@@ -1682,7 +1718,7 @@
         <v>14</v>
       </c>
       <c r="G20" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="H20" t="s">
         <v>127</v>
@@ -1714,24 +1750,24 @@
         <v>14</v>
       </c>
       <c r="G21" t="s">
-        <v>41</v>
+        <v>133</v>
       </c>
       <c r="H21" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="I21" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="J21" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B22" t="s">
-        <v>137</v>
+        <v>83</v>
       </c>
       <c r="C22" t="s">
         <v>12</v>
@@ -1746,7 +1782,7 @@
         <v>14</v>
       </c>
       <c r="G22" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="H22" t="s">
         <v>139</v>
@@ -1778,71 +1814,71 @@
         <v>14</v>
       </c>
       <c r="G23" t="s">
+        <v>47</v>
+      </c>
+      <c r="H23" t="s">
         <v>145</v>
       </c>
-      <c r="H23" t="s">
+      <c r="I23" t="s">
         <v>146</v>
       </c>
-      <c r="I23" t="s">
+      <c r="J23" t="s">
         <v>147</v>
-      </c>
-      <c r="J23" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>148</v>
+      </c>
+      <c r="B24" t="s">
         <v>149</v>
       </c>
-      <c r="B24" t="s">
+      <c r="C24" t="s">
+        <v>12</v>
+      </c>
+      <c r="D24" t="s">
+        <v>12</v>
+      </c>
+      <c r="E24" t="s">
         <v>150</v>
       </c>
-      <c r="C24" t="s">
-        <v>12</v>
-      </c>
-      <c r="D24" t="s">
-        <v>12</v>
-      </c>
-      <c r="E24" t="s">
+      <c r="F24" t="s">
+        <v>14</v>
+      </c>
+      <c r="G24" t="s">
+        <v>47</v>
+      </c>
+      <c r="H24" t="s">
         <v>151</v>
       </c>
-      <c r="F24" t="s">
-        <v>14</v>
-      </c>
-      <c r="G24" t="s">
+      <c r="I24" t="s">
         <v>152</v>
       </c>
-      <c r="H24" t="s">
+      <c r="J24" t="s">
         <v>153</v>
-      </c>
-      <c r="I24" t="s">
-        <v>154</v>
-      </c>
-      <c r="J24" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>154</v>
+      </c>
+      <c r="B25" t="s">
+        <v>155</v>
+      </c>
+      <c r="C25" t="s">
+        <v>12</v>
+      </c>
+      <c r="D25" t="s">
+        <v>12</v>
+      </c>
+      <c r="E25" t="s">
         <v>156</v>
       </c>
-      <c r="B25" t="s">
-        <v>143</v>
-      </c>
-      <c r="C25" t="s">
-        <v>12</v>
-      </c>
-      <c r="D25" t="s">
-        <v>12</v>
-      </c>
-      <c r="E25" t="s">
+      <c r="F25" t="s">
+        <v>14</v>
+      </c>
+      <c r="G25" t="s">
         <v>157</v>
-      </c>
-      <c r="F25" t="s">
-        <v>14</v>
-      </c>
-      <c r="G25" t="s">
-        <v>145</v>
       </c>
       <c r="H25" t="s">
         <v>158</v>
@@ -1859,7 +1895,7 @@
         <v>161</v>
       </c>
       <c r="B26" t="s">
-        <v>150</v>
+        <v>162</v>
       </c>
       <c r="C26" t="s">
         <v>12</v>
@@ -1868,30 +1904,30 @@
         <v>12</v>
       </c>
       <c r="E26" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F26" t="s">
         <v>14</v>
       </c>
       <c r="G26" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="H26" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="I26" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="J26" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B27" t="s">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="C27" t="s">
         <v>12</v>
@@ -1900,13 +1936,13 @@
         <v>12</v>
       </c>
       <c r="E27" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F27" t="s">
         <v>14</v>
       </c>
       <c r="G27" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="H27" t="s">
         <v>170</v>
@@ -1923,103 +1959,103 @@
         <v>173</v>
       </c>
       <c r="B28" t="s">
-        <v>12</v>
+        <v>162</v>
       </c>
       <c r="C28" t="s">
+        <v>12</v>
+      </c>
+      <c r="D28" t="s">
+        <v>12</v>
+      </c>
+      <c r="E28" t="s">
         <v>174</v>
       </c>
-      <c r="D28" t="s">
+      <c r="F28" t="s">
+        <v>14</v>
+      </c>
+      <c r="G28" t="s">
+        <v>164</v>
+      </c>
+      <c r="H28" t="s">
         <v>175</v>
       </c>
-      <c r="E28" t="s">
+      <c r="I28" t="s">
         <v>176</v>
       </c>
-      <c r="F28" t="s">
+      <c r="J28" t="s">
         <v>177</v>
-      </c>
-      <c r="G28" t="s">
-        <v>12</v>
-      </c>
-      <c r="H28" t="s">
-        <v>178</v>
-      </c>
-      <c r="I28" t="s">
-        <v>12</v>
-      </c>
-      <c r="J28" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>178</v>
+      </c>
+      <c r="B29" t="s">
+        <v>179</v>
+      </c>
+      <c r="C29" t="s">
+        <v>12</v>
+      </c>
+      <c r="D29" t="s">
+        <v>12</v>
+      </c>
+      <c r="E29" t="s">
         <v>180</v>
       </c>
-      <c r="B29" t="s">
+      <c r="F29" t="s">
+        <v>14</v>
+      </c>
+      <c r="G29" t="s">
         <v>181</v>
       </c>
-      <c r="C29" t="s">
-        <v>12</v>
-      </c>
-      <c r="D29" t="s">
-        <v>12</v>
-      </c>
-      <c r="E29" t="s">
+      <c r="H29" t="s">
         <v>182</v>
       </c>
-      <c r="F29" t="s">
-        <v>14</v>
-      </c>
-      <c r="G29" t="s">
-        <v>169</v>
-      </c>
-      <c r="H29" t="s">
+      <c r="I29" t="s">
         <v>183</v>
       </c>
-      <c r="I29" t="s">
+      <c r="J29" t="s">
         <v>184</v>
-      </c>
-      <c r="J29" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>185</v>
+      </c>
+      <c r="B30" t="s">
+        <v>12</v>
+      </c>
+      <c r="C30" t="s">
         <v>186</v>
       </c>
-      <c r="B30" t="s">
-        <v>143</v>
-      </c>
-      <c r="C30" t="s">
-        <v>12</v>
-      </c>
       <c r="D30" t="s">
-        <v>12</v>
+        <v>187</v>
       </c>
       <c r="E30" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="F30" t="s">
-        <v>14</v>
+        <v>189</v>
       </c>
       <c r="G30" t="s">
-        <v>145</v>
+        <v>12</v>
       </c>
       <c r="H30" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="I30" t="s">
-        <v>147</v>
+        <v>12</v>
       </c>
       <c r="J30" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B31" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C31" t="s">
         <v>12</v>
@@ -2028,30 +2064,30 @@
         <v>12</v>
       </c>
       <c r="E31" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="F31" t="s">
         <v>14</v>
       </c>
       <c r="G31" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="H31" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="I31" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="J31" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B32" t="s">
-        <v>197</v>
+        <v>155</v>
       </c>
       <c r="C32" t="s">
         <v>12</v>
@@ -2060,19 +2096,19 @@
         <v>12</v>
       </c>
       <c r="E32" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F32" t="s">
         <v>14</v>
       </c>
       <c r="G32" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="H32" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="I32" t="s">
-        <v>200</v>
+        <v>159</v>
       </c>
       <c r="J32" t="s">
         <v>201</v>
@@ -2098,7 +2134,7 @@
         <v>14</v>
       </c>
       <c r="G33" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="H33" t="s">
         <v>205</v>
@@ -2130,7 +2166,7 @@
         <v>14</v>
       </c>
       <c r="G34" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="H34" t="s">
         <v>211</v>
@@ -2140,6 +2176,70 @@
       </c>
       <c r="J34" t="s">
         <v>213</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>214</v>
+      </c>
+      <c r="B35" t="s">
+        <v>215</v>
+      </c>
+      <c r="C35" t="s">
+        <v>12</v>
+      </c>
+      <c r="D35" t="s">
+        <v>12</v>
+      </c>
+      <c r="E35" t="s">
+        <v>216</v>
+      </c>
+      <c r="F35" t="s">
+        <v>14</v>
+      </c>
+      <c r="G35" t="s">
+        <v>181</v>
+      </c>
+      <c r="H35" t="s">
+        <v>217</v>
+      </c>
+      <c r="I35" t="s">
+        <v>218</v>
+      </c>
+      <c r="J35" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>220</v>
+      </c>
+      <c r="B36" t="s">
+        <v>221</v>
+      </c>
+      <c r="C36" t="s">
+        <v>12</v>
+      </c>
+      <c r="D36" t="s">
+        <v>12</v>
+      </c>
+      <c r="E36" t="s">
+        <v>222</v>
+      </c>
+      <c r="F36" t="s">
+        <v>14</v>
+      </c>
+      <c r="G36" t="s">
+        <v>181</v>
+      </c>
+      <c r="H36" t="s">
+        <v>223</v>
+      </c>
+      <c r="I36" t="s">
+        <v>224</v>
+      </c>
+      <c r="J36" t="s">
+        <v>225</v>
       </c>
     </row>
   </sheetData>

</xml_diff>